<commit_message>
Previous Experience is now a single dropdown from the Excel (ExperienceLevel tab)
- Removed Yes/No + Years of Experience number field; one 'Previous Experience'
  dropdown: No, 0-1 year, 1-3 years, 3-5 years, 5-10 years, 10+ years
- New ExperienceLevel tab in options.xlsx + Work Experience section in Settings
- Candidate.experienceLevel replaces hasPreviousExperience/yearsOfExperience

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/options.xlsx
+++ b/public/options.xlsx
@@ -10,6 +10,7 @@
     <sheet name="State" sheetId="5" r:id="rId5"/>
     <sheet name="City" sheetId="6" r:id="rId6"/>
     <sheet name="Qualification" sheetId="7" r:id="rId7"/>
+    <sheet name="ExperienceLevel" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1091,4 +1092,50 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Experience Level</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>0-1 year</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1-3 years</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>3-5 years</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5-10 years</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>10+ years</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>